<commit_message>
y9_mea_01 published: Surface area of right prisms (map flip + JSON export)
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -11572,7 +11572,15 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O140" s="13" t="n">
+        <v>46297</v>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/measurement/y9_mea_01_surface_area_of_right_prisms_v2.html</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">

</xml_diff>

<commit_message>
y9_mea_02 published: Surface area and volume of cylinders (map flip + JSON export)
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -11653,7 +11653,15 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O141" s="13" t="n">
+        <v>46297</v>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/measurement/y9_mea_02_surface_area_and_volume_of_cylinders_v2.html</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">

</xml_diff>

<commit_message>
Mark 10 Y9 lessons Published (map flip + JSON export)
y9_mea_03, 04, 09, 11; y9_spa_01, 04, 06; y9_sta_01, 03; y9_pro_01.
Status, generated date (build-commit date) and URL set; formats copied
from the y9_mea_02 row. Cell diff: only N/O/P on those 10 rows changed.
Published 138 -> 148, Planned 83 -> 73.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JkLiadofJti1Hpn557CtB
</commit_message>
<xml_diff>
--- a/lessonmap.xlsx
+++ b/lessonmap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descriptors" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA Mapping" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Report" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lessons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Descriptors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SA Mapping" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Coverage Report" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lessons'!$A$1:$P$20</definedName>
@@ -11734,7 +11734,15 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O142" s="13" t="n">
+        <v>46297</v>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/measurement/y9_mea_03_optimising_surface_area_and_volume_v2.html</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -11807,7 +11815,15 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O143" s="13" t="n">
+        <v>46298</v>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/measurement/y9_mea_04_introducing_scientific_notation_v2.html</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -12162,7 +12178,15 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O148" s="13" t="n">
+        <v>46299</v>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/measurement/y9_mea_09_absolute_relative_and_percentage_error_v2.html</t>
         </is>
       </c>
     </row>
@@ -12293,7 +12317,15 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O150" s="13" t="n">
+        <v>46300</v>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/measurement/y9_mea_11_modelling_with_direct_proportion_v2.html</t>
         </is>
       </c>
       <c r="Q150" t="inlineStr">
@@ -12429,7 +12461,15 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O152" s="13" t="n">
+        <v>46301</v>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/space/y9_spa_01_naming_sides_in_right_angled_triangles_v2.html</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
@@ -12643,7 +12683,15 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O155" s="13" t="n">
+        <v>46302</v>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/space/y9_spa_04_enlargement_transformation_v2.html</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr">
@@ -12784,7 +12832,15 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O157" s="13" t="n">
+        <v>46303</v>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/space/y9_spa_06_algorithms_for_triangle_properties_v2.html</t>
         </is>
       </c>
       <c r="Q157" t="inlineStr">
@@ -12920,7 +12976,15 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O159" s="13" t="n">
+        <v>46304</v>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/statistics/y9_sta_01_analysing_statistical_reports_v2.html</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr">
@@ -13061,7 +13125,15 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O161" s="13" t="n">
+        <v>46305</v>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/statistics/y9_sta_03_comparing_distributions_visually_v2.html</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
@@ -13343,7 +13415,15 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="O165" s="13" t="n">
+        <v>46306</v>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>https://seager94.github.io/year-9/probability/y9_pro_01_two_step_compound_events_v2.html</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">

</xml_diff>